<commit_message>
feat(server): add payment endpoints, update schemas and services
</commit_message>
<xml_diff>
--- a/server/result.xlsx
+++ b/server/result.xlsx
@@ -427,7 +427,7 @@
     <row ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c s="5" t="inlineStr">
         <is>
-          <t>Tháng: 01/2026</t>
+          <t>Tháng: 03/2026</t>
         </is>
       </c>
       <c s="5"/>
@@ -449,7 +449,7 @@
         </is>
       </c>
       <c s="6" t="n">
-        <v>90000</v>
+        <v>300000</v>
       </c>
       <c s="2"/>
     </row>
@@ -478,7 +478,7 @@
       </c>
       <c s="7" t="inlineStr">
         <is>
-          <t>-70.00 %</t>
+          <t>30000000.00 %</t>
         </is>
       </c>
     </row>
@@ -510,7 +510,7 @@
         </is>
       </c>
       <c s="6" t="n">
-        <v>90000</v>
+        <v>300000</v>
       </c>
     </row>
     <row ht="15.75" x14ac:dyDescent="0.25">
@@ -593,7 +593,7 @@
       </c>
       <c s="7" t="inlineStr">
         <is>
-          <t>9000000.00 %</t>
+          <t>30000000.00 %</t>
         </is>
       </c>
     </row>

</xml_diff>